<commit_message>
feat(redteam): 운영 대화 .xlsx 헤더에 auto-filter 드롭다운 적용
ws.auto_filter.ref = ws.dimensions 한 줄 추가. Excel/Numbers/Google Sheets
모두에서 헤더에 표준 필터 드롭다운이 노출되어 클라이언트가 직접
챗봇/답변 모드/Tier/날짜/검색 결과 수 등으로 필터링·정렬 가능.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/guides/redteam-prod-real-conversations.xlsx
+++ b/docs/guides/redteam-prod-real-conversations.xlsx
@@ -10,7 +10,9 @@
     <sheet name="실제 대화 (dedup)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="요약 통계" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'실제 대화 (dedup)'!$A$1:$U$645</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -61866,6 +61868,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U645"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61903,7 +61906,7 @@
       </c>
       <c r="B2" s="11" t="inlineStr">
         <is>
-          <t>2026-05-04 02:36:40</t>
+          <t>2026-05-04 02:43:15</t>
         </is>
       </c>
     </row>

</xml_diff>